<commit_message>
fix: make workbook checks scenario-aware
</commit_message>
<xml_diff>
--- a/model/nike_valuation_model.xlsx
+++ b/model/nike_valuation_model.xlsx
@@ -6,9 +6,9 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF5FC34-9881-491C-8F00-6D554E402EF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47043F08-6D58-4A50-AA33-EBCEBEE315DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2760" yWindow="2610" windowWidth="11820" windowHeight="10350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -2468,7 +2468,7 @@
     <t>discounting</t>
   </si>
   <si>
-    <t>selected Base</t>
+    <t>selected scenario</t>
   </si>
   <si>
     <t>DCF!E14</t>
@@ -3290,7 +3290,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000000-B918-4C1B-8DEC-8BB9C1075451}"/>
+                <c16:uniqueId val="{00000000-E4C8-4233-A175-F6CAA3770A10}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3305,7 +3305,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-B918-4C1B-8DEC-8BB9C1075451}"/>
+                <c16:uniqueId val="{00000001-E4C8-4233-A175-F6CAA3770A10}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3320,7 +3320,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000002-B918-4C1B-8DEC-8BB9C1075451}"/>
+                <c16:uniqueId val="{00000002-E4C8-4233-A175-F6CAA3770A10}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3335,7 +3335,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-B918-4C1B-8DEC-8BB9C1075451}"/>
+                <c16:uniqueId val="{00000003-E4C8-4233-A175-F6CAA3770A10}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3404,7 +3404,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-B918-4C1B-8DEC-8BB9C1075451}"/>
+              <c16:uniqueId val="{00000004-E4C8-4233-A175-F6CAA3770A10}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -18100,7 +18100,8 @@
         <f>DCF!E24</f>
         <v>52706.027853919441</v>
       </c>
-      <c r="E113" s="5">
+      <c r="E113" s="16">
+        <f>CHOOSE(MATCH(SelectedScenario,ScenarioList,0),DCF!L10,DCF!M10,DCF!N10)</f>
         <v>52706.027853919441</v>
       </c>
       <c r="F113" s="16">
@@ -18132,8 +18133,9 @@
         <f>DCF!E41</f>
         <v>4815.2741252490614</v>
       </c>
-      <c r="E114" s="5">
-        <v>4815.2741252490596</v>
+      <c r="E114" s="16">
+        <f>CHOOSE(MATCH(SelectedScenario,ScenarioList,0),DCF!L20,DCF!M20,DCF!N20)</f>
+        <v>4815.2741252490614</v>
       </c>
       <c r="F114" s="16">
         <f t="shared" si="6"/>
@@ -18164,8 +18166,9 @@
         <f>DCF!E45</f>
         <v>80422.869323639738</v>
       </c>
-      <c r="E115" s="5">
-        <v>80422.869323639708</v>
+      <c r="E115" s="16">
+        <f>CHOOSE(MATCH(SelectedScenario,ScenarioList,0),DCF!L22,DCF!M22,DCF!N22)</f>
+        <v>80422.869323639738</v>
       </c>
       <c r="F115" s="16">
         <f t="shared" si="6"/>
@@ -18196,7 +18199,8 @@
         <f>DCF!E52</f>
         <v>69893.934953875854</v>
       </c>
-      <c r="E116" s="5">
+      <c r="E116" s="16">
+        <f>CHOOSE(MATCH(SelectedScenario,ScenarioList,0),DCF!L24,DCF!M24,DCF!N24)</f>
         <v>69893.934953875854</v>
       </c>
       <c r="F116" s="16">
@@ -18228,7 +18232,8 @@
         <f>DCF!E57</f>
         <v>70978.634953875851</v>
       </c>
-      <c r="E117" s="5">
+      <c r="E117" s="16">
+        <f>CHOOSE(MATCH(SelectedScenario,ScenarioList,0),DCF!L25,DCF!M25,DCF!N25)</f>
         <v>70978.634953875851</v>
       </c>
       <c r="F117" s="16">
@@ -18292,8 +18297,9 @@
         <f>DCF!E60</f>
         <v>47.845431081496429</v>
       </c>
-      <c r="E119" s="5">
-        <v>47.845431081496443</v>
+      <c r="E119" s="16">
+        <f>CHOOSE(MATCH(SelectedScenario,ScenarioList,0),DCF!L27,DCF!M27,DCF!N27)</f>
+        <v>47.845431081496429</v>
       </c>
       <c r="F119" s="16">
         <f t="shared" si="6"/>

</xml_diff>